<commit_message>
adding august 2026 data and model
</commit_message>
<xml_diff>
--- a/model/model_LEI/code/Komposit_LEI_Ketenagakerjaan.xlsx
+++ b/model/model_LEI/code/Komposit_LEI_Ketenagakerjaan.xlsx
@@ -1964,13 +1964,13 @@
         <v>146542264</v>
       </c>
       <c r="E50" t="n">
-        <v>1419.87</v>
+        <v>1423.86</v>
       </c>
       <c r="F50" t="n">
-        <v>31.8199999999999</v>
+        <v>35.8099999999999</v>
       </c>
       <c r="G50" t="n">
-        <v>32.27</v>
+        <v>32.94</v>
       </c>
       <c r="H50" t="n">
         <v>100.04</v>
@@ -1993,13 +1993,13 @@
         <v>146542264</v>
       </c>
       <c r="E51" t="n">
-        <v>1459.91</v>
+        <v>1463.57</v>
       </c>
       <c r="F51" t="n">
-        <v>40.0400000000002</v>
+        <v>39.71</v>
       </c>
       <c r="G51" t="n">
-        <v>31.48</v>
+        <v>32.09</v>
       </c>
       <c r="H51" t="n">
         <v>100.16</v>
@@ -2022,13 +2022,13 @@
         <v>146542264</v>
       </c>
       <c r="E52" t="n">
-        <v>1508.11</v>
+        <v>1513.85</v>
       </c>
       <c r="F52" t="n">
-        <v>48.1999999999998</v>
+        <v>50.28</v>
       </c>
       <c r="G52" t="n">
-        <v>31.9</v>
+        <v>32.86</v>
       </c>
       <c r="H52" t="n">
         <v>100.1</v>
@@ -2051,13 +2051,13 @@
         <v>146542264</v>
       </c>
       <c r="E53" t="n">
-        <v>1563.31</v>
+        <v>1571.59</v>
       </c>
       <c r="F53" t="n">
-        <v>55.2</v>
+        <v>57.74</v>
       </c>
       <c r="G53" t="n">
-        <v>33.32</v>
+        <v>34.7</v>
       </c>
       <c r="H53" t="n">
         <v>100.57</v>
@@ -2080,13 +2080,13 @@
         <v>146542264</v>
       </c>
       <c r="E54" t="n">
-        <v>1633.07</v>
+        <v>1648.03</v>
       </c>
       <c r="F54" t="n">
-        <v>69.76</v>
+        <v>76.44</v>
       </c>
       <c r="G54" t="n">
-        <v>41.34</v>
+        <v>43.83</v>
       </c>
       <c r="H54" t="n">
         <v>101.39</v>
@@ -2109,13 +2109,13 @@
         <v>146542264</v>
       </c>
       <c r="E55" t="n">
-        <v>1672.81</v>
+        <v>1705.91</v>
       </c>
       <c r="F55" t="n">
-        <v>39.74</v>
+        <v>57.8800000000001</v>
       </c>
       <c r="G55" t="n">
-        <v>47.46</v>
+        <v>52.98</v>
       </c>
       <c r="H55" t="n">
         <v>101.93</v>
@@ -2138,13 +2138,13 @@
         <v>146542264</v>
       </c>
       <c r="E56" t="n">
-        <v>1676.57</v>
+        <v>1734.65</v>
       </c>
       <c r="F56" t="n">
-        <v>3.75999999999999</v>
+        <v>28.74</v>
       </c>
       <c r="G56" t="n">
-        <v>42.78</v>
+        <v>51.8</v>
       </c>
       <c r="H56" t="n">
         <v>101.63</v>
@@ -2167,13 +2167,13 @@
         <v>146542264</v>
       </c>
       <c r="E57" t="n">
-        <v>1676.57</v>
+        <v>1742.25</v>
       </c>
       <c r="F57" t="n">
-        <v>0</v>
+        <v>7.59999999999991</v>
       </c>
       <c r="G57" t="n">
-        <v>36.11</v>
+        <v>46.45</v>
       </c>
       <c r="H57" t="n">
         <v>101.9</v>
@@ -3349,7 +3349,7 @@
         <v>2561329</v>
       </c>
       <c r="F50" t="n">
-        <v>772.36</v>
+        <v>999.86</v>
       </c>
       <c r="G50" t="n">
         <v>98.83</v>
@@ -3372,7 +3372,7 @@
         <v>2561329</v>
       </c>
       <c r="F51" t="n">
-        <v>788.85</v>
+        <v>999.86</v>
       </c>
       <c r="G51" t="n">
         <v>98.83</v>
@@ -3395,7 +3395,7 @@
         <v>2561329</v>
       </c>
       <c r="F52" t="n">
-        <v>802.5</v>
+        <v>1014.08</v>
       </c>
       <c r="G52" t="n">
         <v>98.81</v>
@@ -3418,7 +3418,7 @@
         <v>2561329</v>
       </c>
       <c r="F53" t="n">
-        <v>843.45</v>
+        <v>1056.74</v>
       </c>
       <c r="G53" t="n">
         <v>99.29</v>
@@ -3441,7 +3441,7 @@
         <v>2561329</v>
       </c>
       <c r="F54" t="n">
-        <v>864.5</v>
+        <v>1080.62</v>
       </c>
       <c r="G54" t="n">
         <v>100.11</v>
@@ -3464,7 +3464,7 @@
         <v>2561329</v>
       </c>
       <c r="F55" t="n">
-        <v>869.62</v>
+        <v>1093.14</v>
       </c>
       <c r="G55" t="n">
         <v>100.61</v>
@@ -3487,7 +3487,7 @@
         <v>2561329</v>
       </c>
       <c r="F56" t="n">
-        <v>870.75</v>
+        <v>1098.25</v>
       </c>
       <c r="G56" t="n">
         <v>100.32</v>
@@ -3510,7 +3510,7 @@
         <v>2561329</v>
       </c>
       <c r="F57" t="n">
-        <v>870.75</v>
+        <v>1098.82</v>
       </c>
       <c r="G57" t="n">
         <v>100.6</v>
@@ -4637,7 +4637,7 @@
         <v>2701726</v>
       </c>
       <c r="F106" t="n">
-        <v>152.41</v>
+        <v>152.34</v>
       </c>
       <c r="G106" t="n">
         <v>100.27</v>
@@ -4683,7 +4683,7 @@
         <v>2701726</v>
       </c>
       <c r="F108" t="n">
-        <v>159</v>
+        <v>158.93</v>
       </c>
       <c r="G108" t="n">
         <v>100.3</v>
@@ -4706,7 +4706,7 @@
         <v>2701726</v>
       </c>
       <c r="F109" t="n">
-        <v>162.77</v>
+        <v>163.18</v>
       </c>
       <c r="G109" t="n">
         <v>100.78</v>
@@ -4729,7 +4729,7 @@
         <v>2701726</v>
       </c>
       <c r="F110" t="n">
-        <v>165.45</v>
+        <v>166.07</v>
       </c>
       <c r="G110" t="n">
         <v>101.61</v>
@@ -4752,7 +4752,7 @@
         <v>2701726</v>
       </c>
       <c r="F111" t="n">
-        <v>166.41</v>
+        <v>167.99</v>
       </c>
       <c r="G111" t="n">
         <v>102.19</v>
@@ -4775,7 +4775,7 @@
         <v>2701726</v>
       </c>
       <c r="F112" t="n">
-        <v>166.82</v>
+        <v>169.29</v>
       </c>
       <c r="G112" t="n">
         <v>101.89</v>
@@ -4798,7 +4798,7 @@
         <v>2701726</v>
       </c>
       <c r="F113" t="n">
-        <v>166.82</v>
+        <v>169.7</v>
       </c>
       <c r="G113" t="n">
         <v>102.16</v>
@@ -6017,7 +6017,7 @@
         <v>785723</v>
       </c>
       <c r="F166" t="n">
-        <v>407.46</v>
+        <v>408.21</v>
       </c>
       <c r="G166" t="n">
         <v>102</v>
@@ -6040,7 +6040,7 @@
         <v>785723</v>
       </c>
       <c r="F167" t="n">
-        <v>407.96</v>
+        <v>410.22</v>
       </c>
       <c r="G167" t="n">
         <v>102.53</v>
@@ -6063,7 +6063,7 @@
         <v>785723</v>
       </c>
       <c r="F168" t="n">
-        <v>407.96</v>
+        <v>410.22</v>
       </c>
       <c r="G168" t="n">
         <v>102.23</v>
@@ -6086,7 +6086,7 @@
         <v>785723</v>
       </c>
       <c r="F169" t="n">
-        <v>407.96</v>
+        <v>410.22</v>
       </c>
       <c r="G169" t="n">
         <v>102.5</v>
@@ -7213,7 +7213,7 @@
         <v>5755926</v>
       </c>
       <c r="F218" t="n">
-        <v>926.91</v>
+        <v>926.89</v>
       </c>
       <c r="G218" t="n">
         <v>100.11</v>
@@ -7236,7 +7236,7 @@
         <v>5755926</v>
       </c>
       <c r="F219" t="n">
-        <v>944.22</v>
+        <v>944.36</v>
       </c>
       <c r="G219" t="n">
         <v>100.21</v>
@@ -7259,7 +7259,7 @@
         <v>5755926</v>
       </c>
       <c r="F220" t="n">
-        <v>959.19</v>
+        <v>959.5</v>
       </c>
       <c r="G220" t="n">
         <v>99.96</v>
@@ -7282,7 +7282,7 @@
         <v>5755926</v>
       </c>
       <c r="F221" t="n">
-        <v>991.52</v>
+        <v>993.21</v>
       </c>
       <c r="G221" t="n">
         <v>100.42</v>
@@ -7305,7 +7305,7 @@
         <v>5755926</v>
       </c>
       <c r="F222" t="n">
-        <v>1010.83</v>
+        <v>1014.59</v>
       </c>
       <c r="G222" t="n">
         <v>101.28</v>
@@ -7328,7 +7328,7 @@
         <v>5755926</v>
       </c>
       <c r="F223" t="n">
-        <v>1023.33</v>
+        <v>1037.47</v>
       </c>
       <c r="G223" t="n">
         <v>101.81</v>
@@ -7351,7 +7351,7 @@
         <v>5755926</v>
       </c>
       <c r="F224" t="n">
-        <v>1024.33</v>
+        <v>1058.08</v>
       </c>
       <c r="G224" t="n">
         <v>101.48</v>
@@ -7374,7 +7374,7 @@
         <v>5755926</v>
       </c>
       <c r="F225" t="n">
-        <v>1024.33</v>
+        <v>1060.89</v>
       </c>
       <c r="G225" t="n">
         <v>101.76</v>
@@ -8547,7 +8547,7 @@
         <v>1115334</v>
       </c>
       <c r="F276" t="n">
-        <v>1386.87</v>
+        <v>1392.41</v>
       </c>
       <c r="G276" t="n">
         <v>99.7</v>
@@ -8570,7 +8570,7 @@
         <v>1115334</v>
       </c>
       <c r="F277" t="n">
-        <v>1600.81</v>
+        <v>1606.34</v>
       </c>
       <c r="G277" t="n">
         <v>100.17</v>
@@ -8593,7 +8593,7 @@
         <v>1115334</v>
       </c>
       <c r="F278" t="n">
-        <v>1624.78</v>
+        <v>1630.31</v>
       </c>
       <c r="G278" t="n">
         <v>100.99</v>
@@ -8616,7 +8616,7 @@
         <v>1115334</v>
       </c>
       <c r="F279" t="n">
-        <v>1624.78</v>
+        <v>1648.76</v>
       </c>
       <c r="G279" t="n">
         <v>101.2</v>
@@ -8639,7 +8639,7 @@
         <v>1115334</v>
       </c>
       <c r="F280" t="n">
-        <v>1645.07</v>
+        <v>1680.11</v>
       </c>
       <c r="G280" t="n">
         <v>100.91</v>
@@ -8662,7 +8662,7 @@
         <v>1115334</v>
       </c>
       <c r="F281" t="n">
-        <v>1645.07</v>
+        <v>1683.8</v>
       </c>
       <c r="G281" t="n">
         <v>101.19</v>
@@ -9812,7 +9812,7 @@
         <v>2200071</v>
       </c>
       <c r="F331" t="n">
-        <v>3628.81</v>
+        <v>3630.52</v>
       </c>
       <c r="G331" t="n">
         <v>100.16</v>
@@ -9835,7 +9835,7 @@
         <v>2200071</v>
       </c>
       <c r="F332" t="n">
-        <v>3656.84</v>
+        <v>3659.7</v>
       </c>
       <c r="G332" t="n">
         <v>100.11</v>
@@ -9858,7 +9858,7 @@
         <v>2200071</v>
       </c>
       <c r="F333" t="n">
-        <v>3702.61</v>
+        <v>3708.33</v>
       </c>
       <c r="G333" t="n">
         <v>100.58</v>
@@ -9881,7 +9881,7 @@
         <v>2200071</v>
       </c>
       <c r="F334" t="n">
-        <v>3739.22</v>
+        <v>3746.09</v>
       </c>
       <c r="G334" t="n">
         <v>101.44</v>
@@ -9904,7 +9904,7 @@
         <v>2200071</v>
       </c>
       <c r="F335" t="n">
-        <v>3752.38</v>
+        <v>3778.13</v>
       </c>
       <c r="G335" t="n">
         <v>101.97</v>
@@ -9927,7 +9927,7 @@
         <v>2200071</v>
       </c>
       <c r="F336" t="n">
-        <v>3757.53</v>
+        <v>3809.59</v>
       </c>
       <c r="G336" t="n">
         <v>101.66</v>
@@ -9950,7 +9950,7 @@
         <v>2200071</v>
       </c>
       <c r="F337" t="n">
-        <v>3757.53</v>
+        <v>3816.46</v>
       </c>
       <c r="G337" t="n">
         <v>101.93</v>
@@ -11077,7 +11077,7 @@
         <v>5128464</v>
       </c>
       <c r="F386" t="n">
-        <v>1577.62</v>
+        <v>1577.73</v>
       </c>
       <c r="G386" t="n">
         <v>99.88</v>
@@ -11100,7 +11100,7 @@
         <v>5128464</v>
       </c>
       <c r="F387" t="n">
-        <v>1609.87</v>
+        <v>1610.26</v>
       </c>
       <c r="G387" t="n">
         <v>99.94</v>
@@ -11123,7 +11123,7 @@
         <v>5128464</v>
       </c>
       <c r="F388" t="n">
-        <v>1640.45</v>
+        <v>1642.17</v>
       </c>
       <c r="G388" t="n">
         <v>99.88</v>
@@ -11146,7 +11146,7 @@
         <v>5128464</v>
       </c>
       <c r="F389" t="n">
-        <v>1676.2</v>
+        <v>1680.36</v>
       </c>
       <c r="G389" t="n">
         <v>100.36</v>
@@ -11169,7 +11169,7 @@
         <v>5128464</v>
       </c>
       <c r="F390" t="n">
-        <v>1706.01</v>
+        <v>1715</v>
       </c>
       <c r="G390" t="n">
         <v>101.19</v>
@@ -11192,7 +11192,7 @@
         <v>5128464</v>
       </c>
       <c r="F391" t="n">
-        <v>1721.66</v>
+        <v>1741.81</v>
       </c>
       <c r="G391" t="n">
         <v>101.72</v>
@@ -11215,7 +11215,7 @@
         <v>5128464</v>
       </c>
       <c r="F392" t="n">
-        <v>1724.71</v>
+        <v>1762.68</v>
       </c>
       <c r="G392" t="n">
         <v>101.44</v>
@@ -11238,7 +11238,7 @@
         <v>5128464</v>
       </c>
       <c r="F393" t="n">
-        <v>1724.71</v>
+        <v>1764.12</v>
       </c>
       <c r="G393" t="n">
         <v>101.71</v>
@@ -12434,7 +12434,7 @@
         <v>633263</v>
       </c>
       <c r="F445" t="n">
-        <v>291.3</v>
+        <v>291.59</v>
       </c>
       <c r="G445" t="n">
         <v>99.82</v>
@@ -12457,7 +12457,7 @@
         <v>633263</v>
       </c>
       <c r="F446" t="n">
-        <v>292.18</v>
+        <v>293.05</v>
       </c>
       <c r="G446" t="n">
         <v>100.6</v>
@@ -12480,7 +12480,7 @@
         <v>633263</v>
       </c>
       <c r="F447" t="n">
-        <v>292.18</v>
+        <v>293.93</v>
       </c>
       <c r="G447" t="n">
         <v>100.61</v>
@@ -12503,7 +12503,7 @@
         <v>633263</v>
       </c>
       <c r="F448" t="n">
-        <v>292.18</v>
+        <v>293.93</v>
       </c>
       <c r="G448" t="n">
         <v>100.34</v>
@@ -12526,7 +12526,7 @@
         <v>633263</v>
       </c>
       <c r="F449" t="n">
-        <v>292.18</v>
+        <v>294.22</v>
       </c>
       <c r="G449" t="n">
         <v>100.61</v>
@@ -13676,7 +13676,7 @@
         <v>1851864</v>
       </c>
       <c r="F499" t="n">
-        <v>783.86</v>
+        <v>783.33</v>
       </c>
       <c r="G499" t="n">
         <v>99.97</v>
@@ -13722,7 +13722,7 @@
         <v>1851864</v>
       </c>
       <c r="F501" t="n">
-        <v>870.61</v>
+        <v>872.19</v>
       </c>
       <c r="G501" t="n">
         <v>100.4</v>
@@ -13745,7 +13745,7 @@
         <v>1851864</v>
       </c>
       <c r="F502" t="n">
-        <v>890.18</v>
+        <v>895.46</v>
       </c>
       <c r="G502" t="n">
         <v>101.23</v>
@@ -13768,7 +13768,7 @@
         <v>1851864</v>
       </c>
       <c r="F503" t="n">
-        <v>1111.79</v>
+        <v>1123.96</v>
       </c>
       <c r="G503" t="n">
         <v>101.76</v>
@@ -13791,7 +13791,7 @@
         <v>1851864</v>
       </c>
       <c r="F504" t="n">
-        <v>1114.97</v>
+        <v>1134.54</v>
       </c>
       <c r="G504" t="n">
         <v>101.46</v>
@@ -13814,7 +13814,7 @@
         <v>1851864</v>
       </c>
       <c r="F505" t="n">
-        <v>1114.97</v>
+        <v>1136.65</v>
       </c>
       <c r="G505" t="n">
         <v>101.72</v>
@@ -14941,7 +14941,7 @@
         <v>24506852</v>
       </c>
       <c r="F554" t="n">
-        <v>941.78</v>
+        <v>941.8</v>
       </c>
       <c r="G554" t="n">
         <v>100.24</v>
@@ -14964,7 +14964,7 @@
         <v>24506852</v>
       </c>
       <c r="F555" t="n">
-        <v>974.42</v>
+        <v>974.53</v>
       </c>
       <c r="G555" t="n">
         <v>100.29</v>
@@ -14987,7 +14987,7 @@
         <v>24506852</v>
       </c>
       <c r="F556" t="n">
-        <v>1000.81</v>
+        <v>1001.36</v>
       </c>
       <c r="G556" t="n">
         <v>100.25</v>
@@ -15010,7 +15010,7 @@
         <v>24506852</v>
       </c>
       <c r="F557" t="n">
-        <v>1026.2</v>
+        <v>1028.7</v>
       </c>
       <c r="G557" t="n">
         <v>100.71</v>
@@ -15033,7 +15033,7 @@
         <v>24506852</v>
       </c>
       <c r="F558" t="n">
-        <v>1052.89</v>
+        <v>1057.7</v>
       </c>
       <c r="G558" t="n">
         <v>101.54</v>
@@ -15056,7 +15056,7 @@
         <v>24506852</v>
       </c>
       <c r="F559" t="n">
-        <v>1072.37</v>
+        <v>1086.97</v>
       </c>
       <c r="G559" t="n">
         <v>102.07</v>
@@ -15079,7 +15079,7 @@
         <v>24506852</v>
       </c>
       <c r="F560" t="n">
-        <v>1074.01</v>
+        <v>1107.16</v>
       </c>
       <c r="G560" t="n">
         <v>101.77</v>
@@ -15102,7 +15102,7 @@
         <v>24506852</v>
       </c>
       <c r="F561" t="n">
-        <v>1074.01</v>
+        <v>1109.44</v>
       </c>
       <c r="G561" t="n">
         <v>102.03</v>
@@ -16252,7 +16252,7 @@
         <v>21295797</v>
       </c>
       <c r="F611" t="n">
-        <v>2627.73</v>
+        <v>2627.91</v>
       </c>
       <c r="G611" t="n">
         <v>100.42</v>
@@ -16275,7 +16275,7 @@
         <v>21295797</v>
       </c>
       <c r="F612" t="n">
-        <v>2649.06</v>
+        <v>2649.99</v>
       </c>
       <c r="G612" t="n">
         <v>100.29</v>
@@ -16298,7 +16298,7 @@
         <v>21295797</v>
       </c>
       <c r="F613" t="n">
-        <v>2692.53</v>
+        <v>2695.71</v>
       </c>
       <c r="G613" t="n">
         <v>100.73</v>
@@ -16321,7 +16321,7 @@
         <v>21295797</v>
       </c>
       <c r="F614" t="n">
-        <v>2745.35</v>
+        <v>2755.46</v>
       </c>
       <c r="G614" t="n">
         <v>101.58</v>
@@ -16344,7 +16344,7 @@
         <v>21295797</v>
       </c>
       <c r="F615" t="n">
-        <v>2759.63</v>
+        <v>2788.7</v>
       </c>
       <c r="G615" t="n">
         <v>102.16</v>
@@ -16367,7 +16367,7 @@
         <v>21295797</v>
       </c>
       <c r="F616" t="n">
-        <v>2762.19</v>
+        <v>2852.87</v>
       </c>
       <c r="G616" t="n">
         <v>101.85</v>
@@ -16390,7 +16390,7 @@
         <v>21295797</v>
       </c>
       <c r="F617" t="n">
-        <v>2762.19</v>
+        <v>2867.9</v>
       </c>
       <c r="G617" t="n">
         <v>102.13</v>
@@ -17517,7 +17517,7 @@
         <v>23801034</v>
       </c>
       <c r="F666" t="n">
-        <v>488.18</v>
+        <v>488.28</v>
       </c>
       <c r="G666" t="n">
         <v>99.61</v>
@@ -17540,7 +17540,7 @@
         <v>23801034</v>
       </c>
       <c r="F667" t="n">
-        <v>503.37</v>
+        <v>503.52</v>
       </c>
       <c r="G667" t="n">
         <v>99.68</v>
@@ -17563,7 +17563,7 @@
         <v>23801034</v>
       </c>
       <c r="F668" t="n">
-        <v>523.66</v>
+        <v>524.24</v>
       </c>
       <c r="G668" t="n">
         <v>99.66</v>
@@ -17586,7 +17586,7 @@
         <v>23801034</v>
       </c>
       <c r="F669" t="n">
-        <v>543.54</v>
+        <v>544.95</v>
       </c>
       <c r="G669" t="n">
         <v>100.13</v>
@@ -17609,7 +17609,7 @@
         <v>23801034</v>
       </c>
       <c r="F670" t="n">
-        <v>555.06</v>
+        <v>557.74</v>
       </c>
       <c r="G670" t="n">
         <v>100.98</v>
@@ -17632,7 +17632,7 @@
         <v>23801034</v>
       </c>
       <c r="F671" t="n">
-        <v>590.12</v>
+        <v>597.14</v>
       </c>
       <c r="G671" t="n">
         <v>101.54</v>
@@ -17655,7 +17655,7 @@
         <v>23801034</v>
       </c>
       <c r="F672" t="n">
-        <v>592.74</v>
+        <v>605.02</v>
       </c>
       <c r="G672" t="n">
         <v>101.24</v>
@@ -17678,7 +17678,7 @@
         <v>23801034</v>
       </c>
       <c r="F673" t="n">
-        <v>592.74</v>
+        <v>607.71</v>
       </c>
       <c r="G673" t="n">
         <v>101.51</v>
@@ -18805,7 +18805,7 @@
         <v>2930432</v>
       </c>
       <c r="F722" t="n">
-        <v>260.08</v>
+        <v>260.12</v>
       </c>
       <c r="G722" t="n">
         <v>101.08</v>
@@ -18874,7 +18874,7 @@
         <v>2930432</v>
       </c>
       <c r="F725" t="n">
-        <v>274.23</v>
+        <v>274.44</v>
       </c>
       <c r="G725" t="n">
         <v>101.64</v>
@@ -18897,7 +18897,7 @@
         <v>2930432</v>
       </c>
       <c r="F726" t="n">
-        <v>276.33</v>
+        <v>276.87</v>
       </c>
       <c r="G726" t="n">
         <v>102.73</v>
@@ -18920,7 +18920,7 @@
         <v>2930432</v>
       </c>
       <c r="F727" t="n">
-        <v>277.58</v>
+        <v>278.92</v>
       </c>
       <c r="G727" t="n">
         <v>103.24</v>
@@ -18943,7 +18943,7 @@
         <v>2930432</v>
       </c>
       <c r="F728" t="n">
-        <v>278.21</v>
+        <v>280.18</v>
       </c>
       <c r="G728" t="n">
         <v>102.92</v>
@@ -18966,7 +18966,7 @@
         <v>2930432</v>
       </c>
       <c r="F729" t="n">
-        <v>278.21</v>
+        <v>280.22</v>
       </c>
       <c r="G729" t="n">
         <v>103.19</v>
@@ -20093,7 +20093,7 @@
         <v>2153139</v>
       </c>
       <c r="F778" t="n">
-        <v>379.34</v>
+        <v>379.39</v>
       </c>
       <c r="G778" t="n">
         <v>100</v>
@@ -20116,7 +20116,7 @@
         <v>2153139</v>
       </c>
       <c r="F779" t="n">
-        <v>419.46</v>
+        <v>419.62</v>
       </c>
       <c r="G779" t="n">
         <v>100.07</v>
@@ -20139,7 +20139,7 @@
         <v>2153139</v>
       </c>
       <c r="F780" t="n">
-        <v>436.42</v>
+        <v>436.62</v>
       </c>
       <c r="G780" t="n">
         <v>100.01</v>
@@ -20162,7 +20162,7 @@
         <v>2153139</v>
       </c>
       <c r="F781" t="n">
-        <v>442.99</v>
+        <v>443.19</v>
       </c>
       <c r="G781" t="n">
         <v>100.49</v>
@@ -20185,7 +20185,7 @@
         <v>2153139</v>
       </c>
       <c r="F782" t="n">
-        <v>463.25</v>
+        <v>464.33</v>
       </c>
       <c r="G782" t="n">
         <v>101.32</v>
@@ -20208,7 +20208,7 @@
         <v>2153139</v>
       </c>
       <c r="F783" t="n">
-        <v>483.99</v>
+        <v>490.72</v>
       </c>
       <c r="G783" t="n">
         <v>101.85</v>
@@ -20231,7 +20231,7 @@
         <v>2153139</v>
       </c>
       <c r="F784" t="n">
-        <v>485.16</v>
+        <v>497</v>
       </c>
       <c r="G784" t="n">
         <v>101.55</v>
@@ -20254,7 +20254,7 @@
         <v>2153139</v>
       </c>
       <c r="F785" t="n">
-        <v>485.16</v>
+        <v>497.44</v>
       </c>
       <c r="G785" t="n">
         <v>101.82</v>
@@ -21404,7 +21404,7 @@
         <v>1417683</v>
       </c>
       <c r="F835" t="n">
-        <v>2888.68</v>
+        <v>2886.1</v>
       </c>
       <c r="G835" t="n">
         <v>99.18</v>
@@ -21427,7 +21427,7 @@
         <v>1417683</v>
       </c>
       <c r="F836" t="n">
-        <v>3035.36</v>
+        <v>3032.79</v>
       </c>
       <c r="G836" t="n">
         <v>99.14</v>
@@ -21450,7 +21450,7 @@
         <v>1417683</v>
       </c>
       <c r="F837" t="n">
-        <v>3230.94</v>
+        <v>3241.24</v>
       </c>
       <c r="G837" t="n">
         <v>99.33</v>
@@ -21473,7 +21473,7 @@
         <v>1417683</v>
       </c>
       <c r="F838" t="n">
-        <v>3268.26</v>
+        <v>3288.85</v>
       </c>
       <c r="G838" t="n">
         <v>100.15</v>
@@ -21496,7 +21496,7 @@
         <v>1417683</v>
       </c>
       <c r="F839" t="n">
-        <v>3313.29</v>
+        <v>3372.48</v>
       </c>
       <c r="G839" t="n">
         <v>100.66</v>
@@ -21519,7 +21519,7 @@
         <v>1417683</v>
       </c>
       <c r="F840" t="n">
-        <v>3323.59</v>
+        <v>3422.66</v>
       </c>
       <c r="G840" t="n">
         <v>100.42</v>
@@ -21542,7 +21542,7 @@
         <v>1417683</v>
       </c>
       <c r="F841" t="n">
-        <v>3323.59</v>
+        <v>3422.66</v>
       </c>
       <c r="G841" t="n">
         <v>100.69</v>
@@ -22669,7 +22669,7 @@
         <v>1969739</v>
       </c>
       <c r="F890" t="n">
-        <v>231.37</v>
+        <v>231.36</v>
       </c>
       <c r="G890" t="n">
         <v>99.81</v>
@@ -22692,7 +22692,7 @@
         <v>1969739</v>
       </c>
       <c r="F891" t="n">
-        <v>241.58</v>
+        <v>241.64</v>
       </c>
       <c r="G891" t="n">
         <v>99.88</v>
@@ -22715,7 +22715,7 @@
         <v>1969739</v>
       </c>
       <c r="F892" t="n">
-        <v>245.37</v>
+        <v>245.7</v>
       </c>
       <c r="G892" t="n">
         <v>99.84</v>
@@ -22738,7 +22738,7 @@
         <v>1969739</v>
       </c>
       <c r="F893" t="n">
-        <v>251.59</v>
+        <v>252.11</v>
       </c>
       <c r="G893" t="n">
         <v>100.3</v>
@@ -22761,7 +22761,7 @@
         <v>1969739</v>
       </c>
       <c r="F894" t="n">
-        <v>260.46</v>
+        <v>262.03</v>
       </c>
       <c r="G894" t="n">
         <v>101.14</v>
@@ -22784,7 +22784,7 @@
         <v>1969739</v>
       </c>
       <c r="F895" t="n">
-        <v>264.6</v>
+        <v>268.4</v>
       </c>
       <c r="G895" t="n">
         <v>101.66</v>
@@ -22807,7 +22807,7 @@
         <v>1969739</v>
       </c>
       <c r="F896" t="n">
-        <v>264.92</v>
+        <v>269.64</v>
       </c>
       <c r="G896" t="n">
         <v>101.37</v>
@@ -22830,7 +22830,7 @@
         <v>1969739</v>
       </c>
       <c r="F897" t="n">
-        <v>264.92</v>
+        <v>270.11</v>
       </c>
       <c r="G897" t="n">
         <v>101.63</v>
@@ -24026,7 +24026,7 @@
         <v>380572</v>
       </c>
       <c r="F949" t="n">
-        <v>1166.63</v>
+        <v>1166.84</v>
       </c>
       <c r="G949" t="n">
         <v>101.44</v>
@@ -24049,7 +24049,7 @@
         <v>380572</v>
       </c>
       <c r="F950" t="n">
-        <v>1171.15</v>
+        <v>1171.77</v>
       </c>
       <c r="G950" t="n">
         <v>102.25</v>
@@ -24072,7 +24072,7 @@
         <v>380572</v>
       </c>
       <c r="F951" t="n">
-        <v>1171.97</v>
+        <v>1176.08</v>
       </c>
       <c r="G951" t="n">
         <v>102.78</v>
@@ -24095,7 +24095,7 @@
         <v>380572</v>
       </c>
       <c r="F952" t="n">
-        <v>1171.97</v>
+        <v>1176.29</v>
       </c>
       <c r="G952" t="n">
         <v>102.48</v>
@@ -24118,7 +24118,7 @@
         <v>380572</v>
       </c>
       <c r="F953" t="n">
-        <v>1171.97</v>
+        <v>1176.29</v>
       </c>
       <c r="G953" t="n">
         <v>102.76</v>
@@ -25245,7 +25245,7 @@
         <v>1051975</v>
       </c>
       <c r="F1002" t="n">
-        <v>358.07</v>
+        <v>358.01</v>
       </c>
       <c r="G1002" t="n">
         <v>100.57</v>
@@ -25268,7 +25268,7 @@
         <v>1051975</v>
       </c>
       <c r="F1003" t="n">
-        <v>361.38</v>
+        <v>361.32</v>
       </c>
       <c r="G1003" t="n">
         <v>100.64</v>
@@ -25291,7 +25291,7 @@
         <v>1051975</v>
       </c>
       <c r="F1004" t="n">
-        <v>366.1</v>
+        <v>366.21</v>
       </c>
       <c r="G1004" t="n">
         <v>100.52</v>
@@ -25314,7 +25314,7 @@
         <v>1051975</v>
       </c>
       <c r="F1005" t="n">
-        <v>369.52</v>
+        <v>369.74</v>
       </c>
       <c r="G1005" t="n">
         <v>101</v>
@@ -25337,7 +25337,7 @@
         <v>1051975</v>
       </c>
       <c r="F1006" t="n">
-        <v>372.33</v>
+        <v>372.78</v>
       </c>
       <c r="G1006" t="n">
         <v>101.73</v>
@@ -25360,7 +25360,7 @@
         <v>1051975</v>
       </c>
       <c r="F1007" t="n">
-        <v>374.74</v>
+        <v>376.26</v>
       </c>
       <c r="G1007" t="n">
         <v>102.28</v>
@@ -25383,7 +25383,7 @@
         <v>1051975</v>
       </c>
       <c r="F1008" t="n">
-        <v>374.91</v>
+        <v>377.1</v>
       </c>
       <c r="G1008" t="n">
         <v>101.97</v>
@@ -25406,7 +25406,7 @@
         <v>1051975</v>
       </c>
       <c r="F1009" t="n">
-        <v>374.91</v>
+        <v>377.15</v>
       </c>
       <c r="G1009" t="n">
         <v>102.26</v>
@@ -26579,7 +26579,7 @@
         <v>4853377</v>
       </c>
       <c r="F1060" t="n">
-        <v>2010.04</v>
+        <v>2011.65</v>
       </c>
       <c r="G1060" t="n">
         <v>98.9</v>
@@ -26602,7 +26602,7 @@
         <v>4853377</v>
       </c>
       <c r="F1061" t="n">
-        <v>2155.22</v>
+        <v>2164.9</v>
       </c>
       <c r="G1061" t="n">
         <v>99.3</v>
@@ -26625,7 +26625,7 @@
         <v>4853377</v>
       </c>
       <c r="F1062" t="n">
-        <v>2355.26</v>
+        <v>2384.3</v>
       </c>
       <c r="G1062" t="n">
         <v>100.13</v>
@@ -26648,7 +26648,7 @@
         <v>4853377</v>
       </c>
       <c r="F1063" t="n">
-        <v>2389.14</v>
+        <v>2455.28</v>
       </c>
       <c r="G1063" t="n">
         <v>100.64</v>
@@ -26671,7 +26671,7 @@
         <v>4853377</v>
       </c>
       <c r="F1064" t="n">
-        <v>2389.14</v>
+        <v>2490.77</v>
       </c>
       <c r="G1064" t="n">
         <v>100.35</v>
@@ -26694,7 +26694,7 @@
         <v>4853377</v>
       </c>
       <c r="F1065" t="n">
-        <v>2389.14</v>
+        <v>2492.38</v>
       </c>
       <c r="G1065" t="n">
         <v>100.62</v>
@@ -27867,7 +27867,7 @@
         <v>922486</v>
       </c>
       <c r="F1116" t="n">
-        <v>310.36</v>
+        <v>310.8</v>
       </c>
       <c r="G1116" t="n">
         <v>100.84</v>
@@ -27890,7 +27890,7 @@
         <v>922486</v>
       </c>
       <c r="F1117" t="n">
-        <v>312.99</v>
+        <v>313.43</v>
       </c>
       <c r="G1117" t="n">
         <v>101.47</v>
@@ -27913,7 +27913,7 @@
         <v>922486</v>
       </c>
       <c r="F1118" t="n">
-        <v>314.75</v>
+        <v>315.18</v>
       </c>
       <c r="G1118" t="n">
         <v>102.3</v>
@@ -27936,7 +27936,7 @@
         <v>922486</v>
       </c>
       <c r="F1119" t="n">
-        <v>315.18</v>
+        <v>316.94</v>
       </c>
       <c r="G1119" t="n">
         <v>102.8</v>
@@ -27959,7 +27959,7 @@
         <v>922486</v>
       </c>
       <c r="F1120" t="n">
-        <v>315.18</v>
+        <v>319.13</v>
       </c>
       <c r="G1120" t="n">
         <v>102.65</v>
@@ -27982,7 +27982,7 @@
         <v>922486</v>
       </c>
       <c r="F1121" t="n">
-        <v>315.18</v>
+        <v>319.57</v>
       </c>
       <c r="G1121" t="n">
         <v>102.93</v>
@@ -29178,7 +29178,7 @@
         <v>673456</v>
       </c>
       <c r="F1173" t="n">
-        <v>2721.33</v>
+        <v>2733.11</v>
       </c>
       <c r="G1173" t="n">
         <v>100.23</v>
@@ -29201,7 +29201,7 @@
         <v>673456</v>
       </c>
       <c r="F1174" t="n">
-        <v>2786.12</v>
+        <v>2803.79</v>
       </c>
       <c r="G1174" t="n">
         <v>100.44</v>
@@ -29224,7 +29224,7 @@
         <v>673456</v>
       </c>
       <c r="F1175" t="n">
-        <v>2792.01</v>
+        <v>2845.02</v>
       </c>
       <c r="G1175" t="n">
         <v>101.04</v>
@@ -29247,7 +29247,7 @@
         <v>673456</v>
       </c>
       <c r="F1176" t="n">
-        <v>2797.9</v>
+        <v>2933.38</v>
       </c>
       <c r="G1176" t="n">
         <v>100.76</v>
@@ -29270,7 +29270,7 @@
         <v>673456</v>
       </c>
       <c r="F1177" t="n">
-        <v>2797.9</v>
+        <v>2945.16</v>
       </c>
       <c r="G1177" t="n">
         <v>101.04</v>
@@ -30443,7 +30443,7 @@
         <v>3106729</v>
       </c>
       <c r="F1228" t="n">
-        <v>152.14</v>
+        <v>152.03</v>
       </c>
       <c r="G1228" t="n">
         <v>100.46</v>
@@ -30466,7 +30466,7 @@
         <v>3106729</v>
       </c>
       <c r="F1229" t="n">
-        <v>154.49</v>
+        <v>154.61</v>
       </c>
       <c r="G1229" t="n">
         <v>100.95</v>
@@ -30489,7 +30489,7 @@
         <v>3106729</v>
       </c>
       <c r="F1230" t="n">
-        <v>156.49</v>
+        <v>156.96</v>
       </c>
       <c r="G1230" t="n">
         <v>101.78</v>
@@ -30512,7 +30512,7 @@
         <v>3106729</v>
       </c>
       <c r="F1231" t="n">
-        <v>157.55</v>
+        <v>158.84</v>
       </c>
       <c r="G1231" t="n">
         <v>102.32</v>
@@ -30535,7 +30535,7 @@
         <v>3106729</v>
       </c>
       <c r="F1232" t="n">
-        <v>157.67</v>
+        <v>160.37</v>
       </c>
       <c r="G1232" t="n">
         <v>102.01</v>
@@ -30558,7 +30558,7 @@
         <v>3106729</v>
       </c>
       <c r="F1233" t="n">
-        <v>157.67</v>
+        <v>160.37</v>
       </c>
       <c r="G1233" t="n">
         <v>102.28</v>
@@ -31708,7 +31708,7 @@
         <v>2989090</v>
       </c>
       <c r="F1283" t="n">
-        <v>418.14</v>
+        <v>417.36</v>
       </c>
       <c r="G1283" t="n">
         <v>99.92</v>
@@ -31731,7 +31731,7 @@
         <v>2989090</v>
       </c>
       <c r="F1284" t="n">
-        <v>430.65</v>
+        <v>429.87</v>
       </c>
       <c r="G1284" t="n">
         <v>99.88</v>
@@ -31800,7 +31800,7 @@
         <v>2989090</v>
       </c>
       <c r="F1287" t="n">
-        <v>454.88</v>
+        <v>463.48</v>
       </c>
       <c r="G1287" t="n">
         <v>101.71</v>
@@ -31823,7 +31823,7 @@
         <v>2989090</v>
       </c>
       <c r="F1288" t="n">
-        <v>455.66</v>
+        <v>465.82</v>
       </c>
       <c r="G1288" t="n">
         <v>101.41</v>
@@ -31846,7 +31846,7 @@
         <v>2989090</v>
       </c>
       <c r="F1289" t="n">
-        <v>455.66</v>
+        <v>466.6</v>
       </c>
       <c r="G1289" t="n">
         <v>101.68</v>
@@ -33019,7 +33019,7 @@
         <v>434016</v>
       </c>
       <c r="F1340" t="n">
-        <v>1031.99</v>
+        <v>1043.13</v>
       </c>
       <c r="G1340" t="n">
         <v>100.26</v>
@@ -33042,7 +33042,7 @@
         <v>434016</v>
       </c>
       <c r="F1341" t="n">
-        <v>1076.53</v>
+        <v>1087.67</v>
       </c>
       <c r="G1341" t="n">
         <v>100.77</v>
@@ -33065,7 +33065,7 @@
         <v>434016</v>
       </c>
       <c r="F1342" t="n">
-        <v>1195.32</v>
+        <v>1217.6</v>
       </c>
       <c r="G1342" t="n">
         <v>101.59</v>
@@ -33088,7 +33088,7 @@
         <v>434016</v>
       </c>
       <c r="F1343" t="n">
-        <v>1236.16</v>
+        <v>1273.28</v>
       </c>
       <c r="G1343" t="n">
         <v>102.13</v>
@@ -33111,7 +33111,7 @@
         <v>434016</v>
       </c>
       <c r="F1344" t="n">
-        <v>1239.87</v>
+        <v>1280.71</v>
       </c>
       <c r="G1344" t="n">
         <v>101.8</v>
@@ -33134,7 +33134,7 @@
         <v>434016</v>
       </c>
       <c r="F1345" t="n">
-        <v>1239.87</v>
+        <v>1284.42</v>
       </c>
       <c r="G1345" t="n">
         <v>102.08</v>
@@ -34330,7 +34330,7 @@
         <v>288323</v>
       </c>
       <c r="F1397" t="n">
-        <v>441.62</v>
+        <v>447.11</v>
       </c>
       <c r="G1397" t="n">
         <v>100.12</v>
@@ -34353,7 +34353,7 @@
         <v>288323</v>
       </c>
       <c r="F1398" t="n">
-        <v>445.54</v>
+        <v>453.39</v>
       </c>
       <c r="G1398" t="n">
         <v>100.94</v>
@@ -34376,7 +34376,7 @@
         <v>288323</v>
       </c>
       <c r="F1399" t="n">
-        <v>448.68</v>
+        <v>457.31</v>
       </c>
       <c r="G1399" t="n">
         <v>101.47</v>
@@ -34399,7 +34399,7 @@
         <v>288323</v>
       </c>
       <c r="F1400" t="n">
-        <v>449.47</v>
+        <v>459.66</v>
       </c>
       <c r="G1400" t="n">
         <v>101.16</v>
@@ -34422,7 +34422,7 @@
         <v>288323</v>
       </c>
       <c r="F1401" t="n">
-        <v>449.47</v>
+        <v>459.66</v>
       </c>
       <c r="G1401" t="n">
         <v>101.44</v>
@@ -40061,7 +40061,7 @@
         <v>3210929</v>
       </c>
       <c r="F1674" t="n">
-        <v>488.55</v>
+        <v>488.65</v>
       </c>
       <c r="G1674" t="n">
         <v>100.11</v>
@@ -40084,7 +40084,7 @@
         <v>3210929</v>
       </c>
       <c r="F1675" t="n">
-        <v>496.87</v>
+        <v>497.02</v>
       </c>
       <c r="G1675" t="n">
         <v>100.19</v>
@@ -40107,7 +40107,7 @@
         <v>3210929</v>
       </c>
       <c r="F1676" t="n">
-        <v>503.86</v>
+        <v>504.16</v>
       </c>
       <c r="G1676" t="n">
         <v>100.14</v>
@@ -40130,7 +40130,7 @@
         <v>3210929</v>
       </c>
       <c r="F1677" t="n">
-        <v>510.29</v>
+        <v>510.65</v>
       </c>
       <c r="G1677" t="n">
         <v>100.7</v>
@@ -40153,7 +40153,7 @@
         <v>3210929</v>
       </c>
       <c r="F1678" t="n">
-        <v>521.26</v>
+        <v>522.13</v>
       </c>
       <c r="G1678" t="n">
         <v>101.15</v>
@@ -40176,7 +40176,7 @@
         <v>3210929</v>
       </c>
       <c r="F1679" t="n">
-        <v>522.33</v>
+        <v>526.72</v>
       </c>
       <c r="G1679" t="n">
         <v>101.62</v>
@@ -40199,7 +40199,7 @@
         <v>3210929</v>
       </c>
       <c r="F1680" t="n">
-        <v>522.49</v>
+        <v>527.64</v>
       </c>
       <c r="G1680" t="n">
         <v>101.33</v>
@@ -40222,7 +40222,7 @@
         <v>3210929</v>
       </c>
       <c r="F1681" t="n">
-        <v>522.49</v>
+        <v>528</v>
       </c>
       <c r="G1681" t="n">
         <v>101.61</v>
@@ -41395,7 +41395,7 @@
         <v>800433</v>
       </c>
       <c r="F1732" t="n">
-        <v>292.13</v>
+        <v>293.49</v>
       </c>
       <c r="G1732" t="n">
         <v>100.3</v>
@@ -41418,7 +41418,7 @@
         <v>800433</v>
       </c>
       <c r="F1733" t="n">
-        <v>309.87</v>
+        <v>311.24</v>
       </c>
       <c r="G1733" t="n">
         <v>100.76</v>
@@ -41441,7 +41441,7 @@
         <v>800433</v>
       </c>
       <c r="F1734" t="n">
-        <v>322.16</v>
+        <v>327.62</v>
       </c>
       <c r="G1734" t="n">
         <v>101.95</v>
@@ -41464,7 +41464,7 @@
         <v>800433</v>
       </c>
       <c r="F1735" t="n">
-        <v>326.25</v>
+        <v>337.18</v>
       </c>
       <c r="G1735" t="n">
         <v>102.49</v>
@@ -41487,7 +41487,7 @@
         <v>800433</v>
       </c>
       <c r="F1736" t="n">
-        <v>326.25</v>
+        <v>345.37</v>
       </c>
       <c r="G1736" t="n">
         <v>102.17</v>
@@ -41510,7 +41510,7 @@
         <v>800433</v>
       </c>
       <c r="F1737" t="n">
-        <v>326.25</v>
+        <v>345.37</v>
       </c>
       <c r="G1737" t="n">
         <v>102.44</v>
@@ -42660,7 +42660,7 @@
         <v>4759077</v>
       </c>
       <c r="F1787" t="n">
-        <v>1742.08</v>
+        <v>1741.83</v>
       </c>
       <c r="G1787" t="n">
         <v>101.53</v>
@@ -42683,7 +42683,7 @@
         <v>4759077</v>
       </c>
       <c r="F1788" t="n">
-        <v>1798.15</v>
+        <v>1798.9</v>
       </c>
       <c r="G1788" t="n">
         <v>101.52</v>
@@ -42706,7 +42706,7 @@
         <v>4759077</v>
       </c>
       <c r="F1789" t="n">
-        <v>1879.18</v>
+        <v>1883.88</v>
       </c>
       <c r="G1789" t="n">
         <v>102.03</v>
@@ -42729,7 +42729,7 @@
         <v>4759077</v>
       </c>
       <c r="F1790" t="n">
-        <v>2034.57</v>
+        <v>2045.43</v>
       </c>
       <c r="G1790" t="n">
         <v>102.88</v>
@@ -42752,7 +42752,7 @@
         <v>4759077</v>
       </c>
       <c r="F1791" t="n">
-        <v>2058.53</v>
+        <v>2089.65</v>
       </c>
       <c r="G1791" t="n">
         <v>103.4</v>
@@ -42775,7 +42775,7 @@
         <v>4759077</v>
       </c>
       <c r="F1792" t="n">
-        <v>2061.24</v>
+        <v>2113.12</v>
       </c>
       <c r="G1792" t="n">
         <v>103.09</v>
@@ -42798,7 +42798,7 @@
         <v>4759077</v>
       </c>
       <c r="F1793" t="n">
-        <v>2061.24</v>
+        <v>2125.47</v>
       </c>
       <c r="G1793" t="n">
         <v>103.37</v>
@@ -43925,7 +43925,7 @@
         <v>1652846</v>
       </c>
       <c r="F1842" t="n">
-        <v>9912.91</v>
+        <v>9911.58</v>
       </c>
       <c r="G1842" t="n">
         <v>99.9</v>
@@ -43948,7 +43948,7 @@
         <v>1652846</v>
       </c>
       <c r="F1843" t="n">
-        <v>10045.3</v>
+        <v>10042.63</v>
       </c>
       <c r="G1843" t="n">
         <v>99.97</v>
@@ -43994,7 +43994,7 @@
         <v>1652846</v>
       </c>
       <c r="F1845" t="n">
-        <v>10477.23</v>
+        <v>10485.25</v>
       </c>
       <c r="G1845" t="n">
         <v>100.37</v>
@@ -44017,7 +44017,7 @@
         <v>1652846</v>
       </c>
       <c r="F1846" t="n">
-        <v>10812.87</v>
+        <v>10846.3</v>
       </c>
       <c r="G1846" t="n">
         <v>101.19</v>
@@ -44040,7 +44040,7 @@
         <v>1652846</v>
       </c>
       <c r="F1847" t="n">
-        <v>10895.78</v>
+        <v>11002.76</v>
       </c>
       <c r="G1847" t="n">
         <v>101.68</v>
@@ -44063,7 +44063,7 @@
         <v>1652846</v>
       </c>
       <c r="F1848" t="n">
-        <v>10915.84</v>
+        <v>11220.73</v>
       </c>
       <c r="G1848" t="n">
         <v>101.51</v>
@@ -44086,7 +44086,7 @@
         <v>1652846</v>
       </c>
       <c r="F1849" t="n">
-        <v>10915.84</v>
+        <v>11411.95</v>
       </c>
       <c r="G1849" t="n">
         <v>101.79</v>
@@ -45236,7 +45236,7 @@
         <v>1434033</v>
       </c>
       <c r="F1899" t="n">
-        <v>3159.11</v>
+        <v>3158.05</v>
       </c>
       <c r="G1899" t="n">
         <v>100.41</v>
@@ -45282,7 +45282,7 @@
         <v>1434033</v>
       </c>
       <c r="F1901" t="n">
-        <v>3380.45</v>
+        <v>3389.98</v>
       </c>
       <c r="G1901" t="n">
         <v>100.82</v>
@@ -45305,7 +45305,7 @@
         <v>1434033</v>
       </c>
       <c r="F1902" t="n">
-        <v>3558.37</v>
+        <v>3599.67</v>
       </c>
       <c r="G1902" t="n">
         <v>101.64</v>
@@ -45328,7 +45328,7 @@
         <v>1434033</v>
       </c>
       <c r="F1903" t="n">
-        <v>3616.62</v>
+        <v>3693.93</v>
       </c>
       <c r="G1903" t="n">
         <v>102.2</v>
@@ -45351,7 +45351,7 @@
         <v>1434033</v>
       </c>
       <c r="F1904" t="n">
-        <v>3630.39</v>
+        <v>3771.24</v>
       </c>
       <c r="G1904" t="n">
         <v>101.91</v>
@@ -45374,7 +45374,7 @@
         <v>1434033</v>
       </c>
       <c r="F1905" t="n">
-        <v>3630.39</v>
+        <v>3809.36</v>
       </c>
       <c r="G1905" t="n">
         <v>102.18</v>
@@ -46524,7 +46524,7 @@
         <v>1339333</v>
       </c>
       <c r="F1955" t="n">
-        <v>142.28</v>
+        <v>142.19</v>
       </c>
       <c r="G1955" t="n">
         <v>100.05</v>
@@ -46547,7 +46547,7 @@
         <v>1339333</v>
       </c>
       <c r="F1956" t="n">
-        <v>146.55</v>
+        <v>146.46</v>
       </c>
       <c r="G1956" t="n">
         <v>100.01</v>
@@ -46570,7 +46570,7 @@
         <v>1339333</v>
       </c>
       <c r="F1957" t="n">
-        <v>150.9</v>
+        <v>151.32</v>
       </c>
       <c r="G1957" t="n">
         <v>100.49</v>
@@ -46593,7 +46593,7 @@
         <v>1339333</v>
       </c>
       <c r="F1958" t="n">
-        <v>153.41</v>
+        <v>154.33</v>
       </c>
       <c r="G1958" t="n">
         <v>101.33</v>
@@ -46616,7 +46616,7 @@
         <v>1339333</v>
       </c>
       <c r="F1959" t="n">
-        <v>154.25</v>
+        <v>156.42</v>
       </c>
       <c r="G1959" t="n">
         <v>101.86</v>
@@ -46639,7 +46639,7 @@
         <v>1339333</v>
       </c>
       <c r="F1960" t="n">
-        <v>154.33</v>
+        <v>158.01</v>
       </c>
       <c r="G1960" t="n">
         <v>101.55</v>
@@ -46662,7 +46662,7 @@
         <v>1339333</v>
       </c>
       <c r="F1961" t="n">
-        <v>154.33</v>
+        <v>158.1</v>
       </c>
       <c r="G1961" t="n">
         <v>101.82</v>
@@ -47789,7 +47789,7 @@
         <v>3018582</v>
       </c>
       <c r="F2010" t="n">
-        <v>3139.77</v>
+        <v>3142.47</v>
       </c>
       <c r="G2010" t="n">
         <v>98.77</v>
@@ -47812,7 +47812,7 @@
         <v>3018582</v>
       </c>
       <c r="F2011" t="n">
-        <v>3256.91</v>
+        <v>3255.56</v>
       </c>
       <c r="G2011" t="n">
         <v>98.83</v>
@@ -47835,7 +47835,7 @@
         <v>3018582</v>
       </c>
       <c r="F2012" t="n">
-        <v>3427.9</v>
+        <v>3431.94</v>
       </c>
       <c r="G2012" t="n">
         <v>98.79</v>
@@ -47858,7 +47858,7 @@
         <v>3018582</v>
       </c>
       <c r="F2013" t="n">
-        <v>3522.15</v>
+        <v>3528.88</v>
       </c>
       <c r="G2013" t="n">
         <v>99.29</v>
@@ -47881,7 +47881,7 @@
         <v>3018582</v>
       </c>
       <c r="F2014" t="n">
-        <v>3662.17</v>
+        <v>3694.49</v>
       </c>
       <c r="G2014" t="n">
         <v>100.09</v>
@@ -47904,7 +47904,7 @@
         <v>3018582</v>
       </c>
       <c r="F2015" t="n">
-        <v>3756.42</v>
+        <v>3831.82</v>
       </c>
       <c r="G2015" t="n">
         <v>100.58</v>
@@ -47927,7 +47927,7 @@
         <v>3018582</v>
       </c>
       <c r="F2016" t="n">
-        <v>3760.46</v>
+        <v>3877.59</v>
       </c>
       <c r="G2016" t="n">
         <v>100.29</v>
@@ -47950,7 +47950,7 @@
         <v>3018582</v>
       </c>
       <c r="F2017" t="n">
-        <v>3760.46</v>
+        <v>3877.59</v>
       </c>
       <c r="G2017" t="n">
         <v>100.56</v>
@@ -49077,7 +49077,7 @@
         <v>4492574</v>
       </c>
       <c r="F2066" t="n">
-        <v>989.11</v>
+        <v>988.81</v>
       </c>
       <c r="G2066" t="n">
         <v>100.12</v>
@@ -49100,7 +49100,7 @@
         <v>4492574</v>
       </c>
       <c r="F2067" t="n">
-        <v>1042.36</v>
+        <v>1041.44</v>
       </c>
       <c r="G2067" t="n">
         <v>100.19</v>
@@ -49123,7 +49123,7 @@
         <v>4492574</v>
       </c>
       <c r="F2068" t="n">
-        <v>1118.87</v>
+        <v>1118.56</v>
       </c>
       <c r="G2068" t="n">
         <v>100.15</v>
@@ -49146,7 +49146,7 @@
         <v>4492574</v>
       </c>
       <c r="F2069" t="n">
-        <v>1206.4</v>
+        <v>1210.38</v>
       </c>
       <c r="G2069" t="n">
         <v>100.64</v>
@@ -49169,7 +49169,7 @@
         <v>4492574</v>
       </c>
       <c r="F2070" t="n">
-        <v>1238.84</v>
+        <v>1247.41</v>
       </c>
       <c r="G2070" t="n">
         <v>101.46</v>
@@ -49192,7 +49192,7 @@
         <v>4492574</v>
       </c>
       <c r="F2071" t="n">
-        <v>1350.85</v>
+        <v>1454.9</v>
       </c>
       <c r="G2071" t="n">
         <v>101.99</v>
@@ -49215,7 +49215,7 @@
         <v>4492574</v>
       </c>
       <c r="F2072" t="n">
-        <v>1354.52</v>
+        <v>1489.79</v>
       </c>
       <c r="G2072" t="n">
         <v>101.69</v>
@@ -49238,7 +49238,7 @@
         <v>4492574</v>
       </c>
       <c r="F2073" t="n">
-        <v>1354.52</v>
+        <v>1493.15</v>
       </c>
       <c r="G2073" t="n">
         <v>101.96</v>
@@ -50365,7 +50365,7 @@
         <v>7976273</v>
       </c>
       <c r="F2122" t="n">
-        <v>3352.64</v>
+        <v>3351.96</v>
       </c>
       <c r="G2122" t="n">
         <v>101.19</v>
@@ -50411,7 +50411,7 @@
         <v>7976273</v>
       </c>
       <c r="F2124" t="n">
-        <v>3819.8</v>
+        <v>3845.49</v>
       </c>
       <c r="G2124" t="n">
         <v>101.2</v>
@@ -50434,7 +50434,7 @@
         <v>7976273</v>
       </c>
       <c r="F2125" t="n">
-        <v>4113.89</v>
+        <v>4149.05</v>
       </c>
       <c r="G2125" t="n">
         <v>101.67</v>
@@ -50457,7 +50457,7 @@
         <v>7976273</v>
       </c>
       <c r="F2126" t="n">
-        <v>4654.75</v>
+        <v>4733.17</v>
       </c>
       <c r="G2126" t="n">
         <v>102.53</v>
@@ -50480,7 +50480,7 @@
         <v>7976273</v>
       </c>
       <c r="F2127" t="n">
-        <v>4923.82</v>
+        <v>5069.18</v>
       </c>
       <c r="G2127" t="n">
         <v>103.08</v>
@@ -50503,7 +50503,7 @@
         <v>7976273</v>
       </c>
       <c r="F2128" t="n">
-        <v>4949.52</v>
+        <v>5140.17</v>
       </c>
       <c r="G2128" t="n">
         <v>102.78</v>
@@ -50526,7 +50526,7 @@
         <v>7976273</v>
       </c>
       <c r="F2129" t="n">
-        <v>4949.52</v>
+        <v>5159.77</v>
       </c>
       <c r="G2129" t="n">
         <v>103.05</v>

</xml_diff>